<commit_message>
Changed exploratory testing spreadsheet
</commit_message>
<xml_diff>
--- a/docs/ExploratoryTesting.xlsx
+++ b/docs/ExploratoryTesting.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="72">
   <si>
     <t xml:space="preserve">Test</t>
   </si>
@@ -53,6 +53,9 @@
     <t xml:space="preserve">Concurrent restocks (race conditions) </t>
   </si>
   <si>
+    <t xml:space="preserve">Large string names</t>
+  </si>
+  <si>
     <t xml:space="preserve">Large quantity 
 values / integer overflow  </t>
   </si>
@@ -76,6 +79,12 @@
   </si>
   <si>
     <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (whitelabel crash)</t>
   </si>
   <si>
     <t xml:space="preserve">Setup</t>
@@ -117,9 +126,13 @@
 (threads or scripts) </t>
   </si>
   <si>
-    <t xml:space="preserve">Restock with very 
-large quantity
-(Integer.MAX_VALUE) </t>
+    <t xml:space="preserve">Input a long text paragraph into the 
+Product Name field and click Save. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input an overflow value exceeding a
+ 32-bit integer
+ Into the quantity field. </t>
   </si>
   <si>
     <t xml:space="preserve">Start app and open /h2-console
@@ -129,13 +142,13 @@
     <t xml:space="preserve">Offchart</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes </t>
-  </si>
-  <si>
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
     <t xml:space="preserve">No (covered by tests) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No </t>
   </si>
   <si>
     <t xml:space="preserve">Note</t>
@@ -153,8 +166,8 @@
   </si>
   <si>
     <t xml:space="preserve">Service throws IllegalStateException; 
-controller displays error; 
- Consider clearer error page </t>
+controller displays clear top-level 
+Warning banner on the same page</t>
   </si>
   <si>
     <t xml:space="preserve"> Service throws IllegalArgumentException 
@@ -162,15 +175,16 @@
 Validate request params earlier </t>
   </si>
   <si>
-    <t xml:space="preserve">@Column(unique=true) 
-prevents duplicate at DB 
-level; No friendly UI error
-handling visible </t>
-  </si>
-  <si>
-    <t xml:space="preserve">@Email annotation present: 
- test both server-side 
-validation and UI feedback </t>
+    <t xml:space="preserve">UI displays an inline 
+error message, but it
+ is ambiguous </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handled by client-side 
+browser validation via 
+HTML5 email input type. 
+Form submission is 
+Blocked natively. </t>
   </si>
   <si>
     <t xml:space="preserve">ProductRepository.findProductsBelowMinThreshold() 
@@ -182,13 +196,27 @@
 capacity overshoot in edge cases  </t>
   </si>
   <si>
-    <t xml:space="preserve"> Stock fields are Integer; 
-consider validations and limits </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helpful for manual inspection;
- ensure console disabled in 
-Production </t>
+    <t xml:space="preserve">The backend fails to gracefully handle 
+database column length limitations. 
+Saving a long string returns a
+generic fallback error message
+ Instead of a clean validation alert. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend fails during data
+ binding/parsing, crashing to 
+a Whitelabel 400 Bad Request
+ page. The application leaks 
+framework-level errors instead 
+of handling the type
+ Conversion failure gracefully. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">H2 Console is fully accessible
+ at /h2-console. Verified it 
+connects to an in-memory
+ instance (jdbc:h2:mem:inventorydb). 
+Tables map correctly. </t>
   </si>
   <si>
     <t xml:space="preserve">Next time</t>
@@ -201,15 +229,20 @@
  form-level validation </t>
   </si>
   <si>
-    <t xml:space="preserve">Add unit test for capacity check </t>
+    <t xml:space="preserve">Verify if the UI dynamically calculates 
+the maximum allowed quantity 
+before form submission 
+to prevent the user from clicking 
+The button at all. </t>
   </si>
   <si>
     <t xml:space="preserve">Add negative/injection payload tests </t>
   </si>
   <si>
-    <t xml:space="preserve">Test create-product flow and 
-show user-friendly 
-Duplicate-name message </t>
+    <t xml:space="preserve">Verify backend returns a 
+specific error code 
+and the UI is updated to show only
+ "Product name already exists." </t>
   </si>
   <si>
     <t xml:space="preserve">Add unit tests for 
@@ -223,8 +256,19 @@
 Test or optimistic locking </t>
   </si>
   <si>
-    <t xml:space="preserve">Add tests for large inputs 
-And sanitize inputs on UI and API </t>
+    <t xml:space="preserve">Check the database schema definition
+ to find the exact VARCHAR 
+character limit, then add a frontend 
+validation attribute 
+(maxLength) matching it. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement a global @ControllerAdvice/
+ Exception Handler to catch binding 
+exceptions and return a 
+user-friendly error message 
+on the form. Also, add a max attribute
+ On the HTML5 frontend input. </t>
   </si>
   <si>
     <t xml:space="preserve">Document DB login creds 
@@ -248,12 +292,17 @@
     <t xml:space="preserve">Should 404 be returned for missing entities? </t>
   </si>
   <si>
-    <t xml:space="preserve">Is there a product-creation 
-UI endpoint to test?
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Should email be unique? </t>
+    <t xml:space="preserve">Can we remove 'or database error'
+from the UI message so it
+ Doesn't confuse the 
+End-user? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should email be unique? 
+Also, do we want a custom
+, styled UI error message 
+instead of relying on 
+The native browser popup? </t>
   </si>
   <si>
     <t xml:space="preserve">Business rule: include equals or strictly less? </t>
@@ -262,8 +311,16 @@
     <t xml:space="preserve">Acceptable risk level for concurrent updates? </t>
   </si>
   <si>
+    <t xml:space="preserve">What is the maximum practical
+ business length allowed 
+For a product name? </t>
+  </si>
+  <si>
     <t xml:space="preserve">Is there a max business limit for order
- quantity? </t>
+quantity? If so, shouldn't the backend 
+use a Long or data validation annotations
+ (like@Max) instead of letting the
+ Primitive parser crash? </t>
   </si>
   <si>
     <t xml:space="preserve">Should we disable H2 console 
@@ -351,12 +408,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -490,47 +547,48 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="21.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="23.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="42.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="33.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="29.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="24.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="33.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="29.75"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
@@ -538,216 +596,237 @@
       </c>
       <c r="K1" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="C2" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>15</v>
+      <c r="J2" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="K2" s="0" t="s">
-        <v>16</v>
+        <v>19</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="50" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="B3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="E3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="G3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>27</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="32.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="0" t="s">
-        <v>30</v>
+        <v>33</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>16</v>
+        <v>33</v>
+      </c>
+      <c r="L4" s="0" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="48.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="49.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="69.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>57</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="48.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>61</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>